<commit_message>
Simplify the engine: remove unused code, split each scenario into small steps, name every constant, write the Excel KPI values; results unchanged
</commit_message>
<xml_diff>
--- a/output/sacco_stress_test_report.xlsx
+++ b/output/sacco_stress_test_report.xlsx
@@ -45,8 +45,9 @@
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="00666666"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
@@ -106,10 +107,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -508,7 +510,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Report Date: 17 October 2026</t>
+          <t>Report Date: 19 October 2026</t>
         </is>
       </c>
     </row>
@@ -524,6 +526,18 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>KES 231,864,700</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -536,176 +550,188 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>KES 5,439,466</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>2.35%</t>
+        </is>
+      </c>
+    </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>SCENARIO COMPARISON</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Base Case</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Adverse</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Severely Adverse</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>GDP Growth (%)</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="8" t="n">
         <v>-1.5</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Inflation (%)</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B12" s="8" t="n">
         <v>6.5</v>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="8" t="n">
         <v>10.5</v>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="D12" s="8" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>CBR Rate (%)</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="8" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Unemployment Δ (pp)</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="7" t="n">
+      <c r="D14" s="8" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>KES Depreciation (%)</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="8" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Agricultural Shock (%)</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n">
+      <c r="B16" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="7" t="n">
+      <c r="C16" s="8" t="n">
         <v>-15</v>
       </c>
-      <c r="D16" s="7" t="n">
+      <c r="D16" s="8" t="n">
         <v>-30</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>Total ECL (KES)</t>
         </is>
       </c>
-      <c r="B17" s="9" t="n">
+      <c r="B17" s="10" t="n">
         <v>1813103.44</v>
       </c>
-      <c r="C17" s="9" t="n">
+      <c r="C17" s="10" t="n">
         <v>8081951.5</v>
       </c>
-      <c r="D17" s="10" t="n">
+      <c r="D17" s="11" t="n">
         <v>19270186.27</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Provision Rate</t>
         </is>
       </c>
-      <c r="B18" s="11" t="n">
+      <c r="B18" s="12" t="n">
         <v>0.007819661380106587</v>
       </c>
-      <c r="C18" s="11" t="n">
+      <c r="C18" s="12" t="n">
         <v>0.03485632569338929</v>
       </c>
-      <c r="D18" s="11" t="n">
+      <c r="D18" s="12" t="n">
         <v>0.08310961638403776</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Scenario Probability</t>
         </is>
       </c>
-      <c r="B19" s="12" t="n">
+      <c r="B19" s="13" t="n">
         <v>0.6</v>
       </c>
-      <c r="C19" s="12" t="n">
+      <c r="C19" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="D19" s="12" t="n">
+      <c r="D19" s="13" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -737,401 +763,401 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>BASE CASE — IFRS 9 Staging</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Outstanding (KES)</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>ECL (KES)</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Provision Rate</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Avg PD</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>Avg LGD</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>% of Portfolio</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Stage 1</t>
         </is>
       </c>
-      <c r="B3" s="6" t="n">
+      <c r="B3" s="7" t="n">
         <v>1866</v>
       </c>
-      <c r="C3" s="13" t="n">
+      <c r="C3" s="14" t="n">
         <v>215171500</v>
       </c>
-      <c r="D3" s="13" t="n">
+      <c r="D3" s="14" t="n">
         <v>1294491.18</v>
       </c>
-      <c r="E3" s="11" t="n">
+      <c r="E3" s="12" t="n">
         <v>0.006016090327947706</v>
       </c>
-      <c r="F3" s="11" t="n">
+      <c r="F3" s="12" t="n">
         <v>0.0174663729903537</v>
       </c>
-      <c r="G3" s="11" t="n">
+      <c r="G3" s="12" t="n">
         <v>0.4177123258306537</v>
       </c>
-      <c r="H3" s="11" t="n">
+      <c r="H3" s="12" t="n">
         <v>0.9280045647310694</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Stage 2</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n">
+      <c r="B4" s="7" t="n">
         <v>130</v>
       </c>
-      <c r="C4" s="13" t="n">
+      <c r="C4" s="14" t="n">
         <v>16372400</v>
       </c>
-      <c r="D4" s="13" t="n">
+      <c r="D4" s="14" t="n">
         <v>466448.29</v>
       </c>
-      <c r="E4" s="11" t="n">
+      <c r="E4" s="12" t="n">
         <v>0.02848991534533727</v>
       </c>
-      <c r="F4" s="11" t="n">
+      <c r="F4" s="12" t="n">
         <v>0.0812027076923077</v>
       </c>
-      <c r="G4" s="11" t="n">
+      <c r="G4" s="12" t="n">
         <v>0.52528</v>
       </c>
-      <c r="H4" s="11" t="n">
+      <c r="H4" s="12" t="n">
         <v>0.070611869767153</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Stage 3</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="14" t="n">
         <v>320800</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="14" t="n">
         <v>52163.97</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="12" t="n">
         <v>0.162605891521197</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="12" t="n">
         <v>0.6406999999999999</v>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="G5" s="12" t="n">
         <v>0.4824000000000001</v>
       </c>
-      <c r="H5" s="11" t="n">
+      <c r="H5" s="12" t="n">
         <v>0.001383565501777545</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>ADVERSE — IFRS 9 Staging</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Outstanding (KES)</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>ECL (KES)</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Provision Rate</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Avg PD</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Avg LGD</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>% of Portfolio</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Stage 1</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="7" t="n">
         <v>1866</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="14" t="n">
         <v>215171500</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="14" t="n">
         <v>5912241.24</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="12" t="n">
         <v>0.02747687886174517</v>
       </c>
-      <c r="F9" s="11" t="n">
+      <c r="F9" s="12" t="n">
         <v>0.04928991371918542</v>
       </c>
-      <c r="G9" s="11" t="n">
+      <c r="G9" s="12" t="n">
         <v>0.6398829581993568</v>
       </c>
-      <c r="H9" s="11" t="n">
+      <c r="H9" s="12" t="n">
         <v>0.9280045647310694</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Stage 2</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="7" t="n">
         <v>130</v>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="14" t="n">
         <v>16372400</v>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="14" t="n">
         <v>2017893.17</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="12" t="n">
         <v>0.1232496866678068</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="12" t="n">
         <v>0.2291253692307692</v>
       </c>
-      <c r="G10" s="11" t="n">
+      <c r="G10" s="12" t="n">
         <v>0.7530776923076923</v>
       </c>
-      <c r="H10" s="11" t="n">
+      <c r="H10" s="12" t="n">
         <v>0.070611869767153</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Stage 3</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B11" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="14" t="n">
         <v>320800</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <v>151817.09</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="12" t="n">
         <v>0.4732452930174563</v>
       </c>
-      <c r="F11" s="11" t="n">
+      <c r="F11" s="12" t="n">
         <v>0.99</v>
       </c>
-      <c r="G11" s="11" t="n">
+      <c r="G11" s="12" t="n">
         <v>0.70165</v>
       </c>
-      <c r="H11" s="11" t="n">
+      <c r="H11" s="12" t="n">
         <v>0.001383565501777545</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>SEVERELY ADVERSE — IFRS 9 Staging</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Outstanding (KES)</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>ECL (KES)</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Provision Rate</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Avg PD</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>Avg LGD</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>% of Portfolio</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Stage 1</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B15" s="7" t="n">
         <v>1866</v>
       </c>
-      <c r="C15" s="13" t="n">
+      <c r="C15" s="14" t="n">
         <v>215171500</v>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="14" t="n">
         <v>14250134.55</v>
       </c>
-      <c r="E15" s="11" t="n">
+      <c r="E15" s="12" t="n">
         <v>0.06622686810288538</v>
       </c>
-      <c r="F15" s="11" t="n">
+      <c r="F15" s="12" t="n">
         <v>0.09172203269024654</v>
       </c>
-      <c r="G15" s="11" t="n">
+      <c r="G15" s="12" t="n">
         <v>0.7883400321543409</v>
       </c>
-      <c r="H15" s="11" t="n">
+      <c r="H15" s="12" t="n">
         <v>0.9280045647310694</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Stage 2</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n">
+      <c r="B16" s="7" t="n">
         <v>130</v>
       </c>
-      <c r="C16" s="13" t="n">
+      <c r="C16" s="14" t="n">
         <v>16372400</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D16" s="14" t="n">
         <v>4800566.73</v>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="12" t="n">
         <v>0.293210936087562</v>
       </c>
-      <c r="F16" s="11" t="n">
+      <c r="F16" s="12" t="n">
         <v>0.4262894769230769</v>
       </c>
-      <c r="G16" s="11" t="n">
+      <c r="G16" s="12" t="n">
         <v>0.843096153846154</v>
       </c>
-      <c r="H16" s="11" t="n">
+      <c r="H16" s="12" t="n">
         <v>0.070611869767153</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Stage 3</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n">
+      <c r="B17" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="C17" s="13" t="n">
+      <c r="C17" s="14" t="n">
         <v>320800</v>
       </c>
-      <c r="D17" s="13" t="n">
+      <c r="D17" s="14" t="n">
         <v>219484.99</v>
       </c>
-      <c r="E17" s="11" t="n">
+      <c r="E17" s="12" t="n">
         <v>0.6841801433915212</v>
       </c>
-      <c r="F17" s="11" t="n">
+      <c r="F17" s="12" t="n">
         <v>0.99</v>
       </c>
-      <c r="G17" s="11" t="n">
+      <c r="G17" s="12" t="n">
         <v>0.81375</v>
       </c>
-      <c r="H17" s="11" t="n">
+      <c r="H17" s="12" t="n">
         <v>0.001383565501777545</v>
       </c>
     </row>
@@ -1157,207 +1183,207 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>SECTOR VULNERABILITY — ADVERSE SCENARIO</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Sector</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Loan Count</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Outstanding (KES)</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>ECL (KES)</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Provision Rate</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Agriculture</t>
         </is>
       </c>
-      <c r="B3" s="6" t="n">
+      <c r="B3" s="7" t="n">
         <v>233</v>
       </c>
-      <c r="C3" s="13" t="n">
+      <c r="C3" s="14" t="n">
         <v>24015600</v>
       </c>
-      <c r="D3" s="13" t="n">
+      <c r="D3" s="14" t="n">
         <v>1085603.07</v>
       </c>
-      <c r="E3" s="11" t="n">
+      <c r="E3" s="12" t="n">
         <v>0.04520407859891071</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n">
+      <c r="B4" s="7" t="n">
         <v>222</v>
       </c>
-      <c r="C4" s="13" t="n">
+      <c r="C4" s="14" t="n">
         <v>30187000</v>
       </c>
-      <c r="D4" s="13" t="n">
+      <c r="D4" s="14" t="n">
         <v>1198332.19</v>
       </c>
-      <c r="E4" s="11" t="n">
+      <c r="E4" s="12" t="n">
         <v>0.03969696193725776</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Trade</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="7" t="n">
         <v>214</v>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="14" t="n">
         <v>23891700</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="14" t="n">
         <v>870136.45</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="12" t="n">
         <v>0.03642003080567728</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Transport</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="7" t="n">
         <v>223</v>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="14" t="n">
         <v>23706400</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="14" t="n">
         <v>845589.67</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="12" t="n">
         <v>0.03566925682516114</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Construction</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="7" t="n">
         <v>216</v>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="14" t="n">
         <v>26359900</v>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="14" t="n">
         <v>913825.1800000001</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="12" t="n">
         <v>0.0346672475995736</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="7" t="n">
         <v>232</v>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="14" t="n">
         <v>25133600</v>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="14" t="n">
         <v>821662.95</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="12" t="n">
         <v>0.03269181295158672</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Health</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="7" t="n">
         <v>220</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="14" t="n">
         <v>24039700</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="14" t="n">
         <v>741667.4</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="12" t="n">
         <v>0.03085177435658515</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Manufacturing</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="7" t="n">
         <v>212</v>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="14" t="n">
         <v>28755600</v>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="14" t="n">
         <v>846714.89</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="12" t="n">
         <v>0.02944521727941688</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Services</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B11" s="7" t="n">
         <v>228</v>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="14" t="n">
         <v>25775200</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <v>758419.7</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="12" t="n">
         <v>0.02942439631894224</v>
       </c>
     </row>
@@ -1382,89 +1408,89 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>PROBABILITY-WEIGHTED EXPECTED CREDIT LOSS</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Scenario</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>ECL (KES)</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Probability</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Weighted Contribution (KES)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Base Case</t>
         </is>
       </c>
-      <c r="B4" s="13" t="n">
+      <c r="B4" s="14" t="n">
         <v>1813103.44</v>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="C4" s="13" t="n">
         <v>0.6</v>
       </c>
-      <c r="D4" s="13" t="n">
+      <c r="D4" s="14" t="n">
         <v>1087862.064</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Adverse</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n">
+      <c r="B5" s="14" t="n">
         <v>8081951.5</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="14" t="n">
         <v>2424585.45</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Severely Adverse</t>
         </is>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="14" t="n">
         <v>19270186.27</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="13" t="n">
         <v>0.1</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="14" t="n">
         <v>1927018.627</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>TOTAL WEIGHTED ECL</t>
         </is>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="16" t="n">
         <v>5439466.141</v>
       </c>
     </row>
@@ -1474,7 +1500,7 @@
           <t>Weighted Provision Rate</t>
         </is>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D8" s="17" t="n">
         <v>0.02345965617448452</v>
       </c>
     </row>

</xml_diff>